<commit_message>
dashboard and form updates
</commit_message>
<xml_diff>
--- a/assets/downloadables/DCF_Form_3.xlsx
+++ b/assets/downloadables/DCF_Form_3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Systems\dti_web_app_v2\assets\downloadables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E183ED-1A2E-4B73-A270-92406489C834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F608D449-96AF-497B-96E2-08A4530632F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="form3" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="68">
   <si>
     <t>FORM 3 - BDSP REGISTRY</t>
   </si>
@@ -246,10 +246,13 @@
     <t>Select one (RED,PLATINUM,UNREGISTERED)</t>
   </si>
   <si>
-    <t>Name of BDSP:</t>
-  </si>
-  <si>
     <t>(For organization/firm BDSPs, input the name of BDSP. For individuals, leave it blank)</t>
+  </si>
+  <si>
+    <t>Classiciation</t>
+  </si>
+  <si>
+    <t>(dropdown: BDSP/FSP)</t>
   </si>
 </sst>
 </file>
@@ -365,7 +368,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -492,11 +495,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -621,8 +646,8 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -630,7 +655,16 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -913,157 +947,164 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:AA20"/>
+  <dimension ref="A2:AB20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.5703125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" style="9" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" style="9" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="9" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="28.7109375" style="9" customWidth="1"/>
-    <col min="7" max="7" width="35.5703125" style="9" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" style="9" customWidth="1"/>
-    <col min="9" max="9" width="24.140625" style="9" customWidth="1"/>
-    <col min="10" max="10" width="29.85546875" style="9" customWidth="1"/>
-    <col min="11" max="11" width="34" style="9" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" style="9" customWidth="1"/>
-    <col min="13" max="13" width="24" style="9" customWidth="1"/>
-    <col min="14" max="14" width="30.28515625" style="9" customWidth="1"/>
-    <col min="15" max="15" width="27.5703125" style="9" customWidth="1"/>
-    <col min="16" max="16" width="27.42578125" style="9" customWidth="1"/>
-    <col min="17" max="17" width="27.7109375" style="9" customWidth="1"/>
-    <col min="18" max="18" width="32.42578125" style="9" customWidth="1"/>
-    <col min="19" max="19" width="30.7109375" style="9" customWidth="1"/>
-    <col min="20" max="20" width="31.85546875" style="9" customWidth="1"/>
-    <col min="21" max="21" width="37.140625" style="9" customWidth="1"/>
-    <col min="22" max="22" width="42.42578125" style="9" customWidth="1"/>
-    <col min="23" max="23" width="38.42578125" style="9" customWidth="1"/>
-    <col min="24" max="24" width="38.28515625" style="9" customWidth="1"/>
-    <col min="25" max="25" width="24" style="9" customWidth="1"/>
-    <col min="26" max="26" width="18.5703125" style="9" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="9"/>
+    <col min="2" max="2" width="17" style="9" customWidth="1"/>
+    <col min="3" max="3" width="38.5703125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="26.85546875" style="9" customWidth="1"/>
+    <col min="7" max="7" width="28.7109375" style="9" customWidth="1"/>
+    <col min="8" max="8" width="35.5703125" style="9" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" style="9" customWidth="1"/>
+    <col min="10" max="10" width="24.140625" style="9" customWidth="1"/>
+    <col min="11" max="11" width="29.85546875" style="9" customWidth="1"/>
+    <col min="12" max="12" width="34" style="9" customWidth="1"/>
+    <col min="13" max="13" width="23.7109375" style="9" customWidth="1"/>
+    <col min="14" max="14" width="24" style="9" customWidth="1"/>
+    <col min="15" max="15" width="30.28515625" style="9" customWidth="1"/>
+    <col min="16" max="16" width="27.5703125" style="9" customWidth="1"/>
+    <col min="17" max="17" width="27.42578125" style="9" customWidth="1"/>
+    <col min="18" max="18" width="27.7109375" style="9" customWidth="1"/>
+    <col min="19" max="19" width="32.42578125" style="9" customWidth="1"/>
+    <col min="20" max="20" width="30.7109375" style="9" customWidth="1"/>
+    <col min="21" max="21" width="31.85546875" style="9" customWidth="1"/>
+    <col min="22" max="22" width="37.140625" style="9" customWidth="1"/>
+    <col min="23" max="23" width="42.42578125" style="9" customWidth="1"/>
+    <col min="24" max="24" width="38.42578125" style="9" customWidth="1"/>
+    <col min="25" max="25" width="38.28515625" style="9" customWidth="1"/>
+    <col min="26" max="26" width="24" style="9" customWidth="1"/>
+    <col min="27" max="27" width="18.5703125" style="9" customWidth="1"/>
+    <col min="28" max="16384" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="2"/>
+      <c r="C2" s="1"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="2"/>
+      <c r="G2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="10"/>
       <c r="H2" s="10"/>
       <c r="I2" s="10"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="7"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="3"/>
       <c r="L2" s="7"/>
       <c r="M2" s="7"/>
       <c r="N2" s="7"/>
-      <c r="O2" s="11" t="s">
+      <c r="O2" s="7"/>
+      <c r="P2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="P2" s="12"/>
       <c r="Q2" s="12"/>
       <c r="R2" s="12"/>
       <c r="S2" s="12"/>
-      <c r="T2" s="13" t="s">
+      <c r="T2" s="12"/>
+      <c r="U2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="U2" s="14"/>
       <c r="V2" s="14"/>
       <c r="W2" s="14"/>
       <c r="X2" s="14"/>
       <c r="Y2" s="14"/>
-      <c r="Z2" s="6"/>
-      <c r="AA2" s="8"/>
-    </row>
-    <row r="3" spans="1:27" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="46" t="s">
-        <v>65</v>
+      <c r="Z2" s="14"/>
+      <c r="AA2" s="6"/>
+      <c r="AB2" s="8"/>
+    </row>
+    <row r="3" spans="1:28" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="49" t="s">
+        <v>66</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="51" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="F3" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="G3" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="H3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="I3" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="J3" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="K3" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="15" t="s">
+      <c r="L3" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="17" t="s">
+      <c r="M3" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="18"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="20" t="s">
+      <c r="N3" s="18"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="P3" s="21" t="s">
+      <c r="Q3" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="Q3" s="21" t="s">
+      <c r="R3" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="21" t="s">
+      <c r="S3" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="S3" s="21" t="s">
+      <c r="T3" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T3" s="22" t="s">
+      <c r="U3" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="22" t="s">
+      <c r="V3" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="V3" s="22" t="s">
+      <c r="W3" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="W3" s="22" t="s">
+      <c r="X3" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="X3" s="22" t="s">
+      <c r="Y3" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="Y3" s="22" t="s">
+      <c r="Z3" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="Z3" s="23" t="s">
+      <c r="AA3" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="AA3" s="47"/>
-    </row>
-    <row r="4" spans="1:27" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="49" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="24"/>
+      <c r="AB3" s="47"/>
+    </row>
+    <row r="4" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="52"/>
+      <c r="C4" s="46" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="25"/>
       <c r="E4" s="24"/>
       <c r="F4" s="24"/>
       <c r="G4" s="24"/>
@@ -1071,30 +1112,31 @@
       <c r="I4" s="24"/>
       <c r="J4" s="24"/>
       <c r="K4" s="24"/>
-      <c r="L4" s="4" t="s">
+      <c r="L4" s="24"/>
+      <c r="M4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="N4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N4" s="4" t="s">
+      <c r="O4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="26"/>
-      <c r="P4" s="27"/>
+      <c r="P4" s="26"/>
       <c r="Q4" s="27"/>
       <c r="R4" s="27"/>
       <c r="S4" s="27"/>
-      <c r="T4" s="28"/>
+      <c r="T4" s="27"/>
       <c r="U4" s="28"/>
       <c r="V4" s="28"/>
       <c r="W4" s="28"/>
       <c r="X4" s="28"/>
       <c r="Y4" s="28"/>
-      <c r="Z4" s="29"/>
-      <c r="AA4" s="48"/>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z4" s="28"/>
+      <c r="AA4" s="29"/>
+      <c r="AB4" s="48"/>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="39">
         <v>0</v>
       </c>
@@ -1173,9 +1215,12 @@
       <c r="Z5" s="39">
         <v>25</v>
       </c>
-      <c r="AA5" s="5"/>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AA5" s="39">
+        <v>26</v>
+      </c>
+      <c r="AB5" s="5"/>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1203,8 +1248,9 @@
       <c r="Y6" s="5"/>
       <c r="Z6" s="5"/>
       <c r="AA6" s="5"/>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB6" s="5"/>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -1232,8 +1278,9 @@
       <c r="Y7" s="5"/>
       <c r="Z7" s="5"/>
       <c r="AA7" s="5"/>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB7" s="5"/>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1261,8 +1308,9 @@
       <c r="Y8" s="5"/>
       <c r="Z8" s="5"/>
       <c r="AA8" s="5"/>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB8" s="5"/>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -1290,8 +1338,9 @@
       <c r="Y9" s="5"/>
       <c r="Z9" s="5"/>
       <c r="AA9" s="5"/>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB9" s="5"/>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1319,8 +1368,9 @@
       <c r="Y10" s="5"/>
       <c r="Z10" s="5"/>
       <c r="AA10" s="5"/>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB10" s="5"/>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1348,8 +1398,9 @@
       <c r="Y11" s="5"/>
       <c r="Z11" s="5"/>
       <c r="AA11" s="5"/>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB11" s="5"/>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1377,8 +1428,9 @@
       <c r="Y12" s="5"/>
       <c r="Z12" s="5"/>
       <c r="AA12" s="5"/>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB12" s="5"/>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1406,8 +1458,9 @@
       <c r="Y13" s="5"/>
       <c r="Z13" s="5"/>
       <c r="AA13" s="5"/>
-    </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB13" s="5"/>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1435,8 +1488,9 @@
       <c r="Y14" s="5"/>
       <c r="Z14" s="5"/>
       <c r="AA14" s="5"/>
-    </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB14" s="5"/>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1464,8 +1518,9 @@
       <c r="Y15" s="5"/>
       <c r="Z15" s="5"/>
       <c r="AA15" s="5"/>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB15" s="5"/>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1493,8 +1548,9 @@
       <c r="Y16" s="5"/>
       <c r="Z16" s="5"/>
       <c r="AA16" s="5"/>
-    </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB16" s="5"/>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1522,8 +1578,9 @@
       <c r="Y17" s="5"/>
       <c r="Z17" s="5"/>
       <c r="AA17" s="5"/>
-    </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB17" s="5"/>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1551,8 +1608,9 @@
       <c r="Y18" s="5"/>
       <c r="Z18" s="5"/>
       <c r="AA18" s="5"/>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB18" s="5"/>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1580,8 +1638,9 @@
       <c r="Y19" s="5"/>
       <c r="Z19" s="5"/>
       <c r="AA19" s="5"/>
-    </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB19" s="5"/>
+    </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1609,10 +1668,11 @@
       <c r="Y20" s="5"/>
       <c r="Z20" s="5"/>
       <c r="AA20" s="5"/>
+      <c r="AB20" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="AA3:AA4"/>
+    <mergeCell ref="AB3:AB4"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>